<commit_message>
uVerter copy as KiCad starting point
</commit_message>
<xml_diff>
--- a/Design Notes/20260609 LibreDAB_planning_pack.xlsx
+++ b/Design Notes/20260609 LibreDAB_planning_pack.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId3"/>
@@ -1146,7 +1146,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0"/>
@@ -1155,7 +1155,6 @@
     <numFmt numFmtId="169" formatCode="0.0%"/>
     <numFmt numFmtId="170" formatCode="\£#,##0.00"/>
     <numFmt numFmtId="171" formatCode="0.00"/>
-    <numFmt numFmtId="172" formatCode="General"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -1299,104 +1298,108 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1470,6 +1473,49 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>409320</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>117000</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 1"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="5133240"/>
+          <a:ext cx="11054520" cy="5451120"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1653,159 +1699,159 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B22"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="105"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="105"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="4"/>
+      <c r="B3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
+      <c r="A7" s="4"/>
+      <c r="B7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
-      <c r="B11" s="4"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="4"/>
+      <c r="B12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3"/>
-      <c r="B20" s="4"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3"/>
-      <c r="B22" s="4" t="s">
+      <c r="A22" s="4"/>
+      <c r="B22" s="5" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1817,6 +1863,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1826,400 +1873,400 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C42"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="8" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="9" t="n">
         <v>42</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="10" t="n">
         <v>23.8</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="10" t="n">
         <v>58.8</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="10" t="n">
         <v>400</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="10" t="n">
         <v>800</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="9" t="n">
-        <v>11</v>
-      </c>
-      <c r="C11" s="3" t="s">
+      <c r="B11" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="10" t="n">
         <v>3.7E-006</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="10" t="n">
         <v>0.000146</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="10" t="n">
         <v>0.95</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="9" t="n">
+      <c r="B17" s="10" t="n">
         <v>1.2</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="8" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="11" t="n">
         <f aca="false">$B$11*$B$12</f>
-        <v>11</v>
-      </c>
-      <c r="C20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B21" s="12" t="n">
         <f aca="false">$B$8/$B$11</f>
-        <v>36.3636363636364</v>
-      </c>
-      <c r="C21" s="3" t="s">
+        <v>23.5294117647059</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B22" s="11" t="n">
+      <c r="B22" s="12" t="n">
         <f aca="false">$B$9/$B$5</f>
         <v>19.047619047619</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="4" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="11" t="n">
+      <c r="B23" s="12" t="n">
         <f aca="false">$B$9/($B$16*$B$6)</f>
         <v>35.3825740822645</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="4" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="12" t="n">
+      <c r="B24" s="13" t="n">
         <f aca="false">$B$15*PI()/180</f>
         <v>0.872664625997165</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="4" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B25" s="12" t="n">
+      <c r="B25" s="13" t="n">
         <f aca="false">B24*(1-B24/PI())</f>
         <v>0.630257785442397</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B26" s="13" t="n">
+      <c r="B26" s="14" t="n">
         <f aca="false">$B$5*B21*B25/(2*PI()*$B$10*$B$9)</f>
-        <v>1.91498316498317E-007</v>
-      </c>
-      <c r="C26" s="3" t="s">
+        <v>1.23910675381264E-007</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B27" s="10" t="n">
+      <c r="B27" s="11" t="n">
         <f aca="false">B26*1000000000</f>
-        <v>191.498316498317</v>
-      </c>
-      <c r="C27" s="3" t="s">
+        <v>123.910675381264</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B28" s="11" t="n">
+      <c r="B28" s="12" t="n">
         <f aca="false">B26*$B$11^2*1000000</f>
-        <v>23.1712962962963</v>
-      </c>
-      <c r="C28" s="3" t="s">
+        <v>35.8101851851852</v>
+      </c>
+      <c r="C28" s="4" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
+      <c r="A29" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B29" s="13" t="n">
+      <c r="B29" s="14" t="n">
         <f aca="false">$B$13*$B$12^2</f>
         <v>3.7E-006</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="4" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B30" s="14" t="n">
+      <c r="B30" s="15" t="n">
         <f aca="false">B26/B29</f>
-        <v>0.0517563017563018</v>
-      </c>
-      <c r="C30" s="3" t="s">
+        <v>0.0334893717246659</v>
+      </c>
+      <c r="C30" s="4" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B31" s="12" t="n">
+      <c r="B31" s="13" t="n">
         <f aca="false">$B$8/(4*$B$10*B20*$B$14)</f>
-        <v>0.062266500622665</v>
-      </c>
-      <c r="C31" s="3" t="s">
+        <v>0.040290088638195</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="11" t="n">
         <f aca="false">B31*1000</f>
-        <v>62.266500622665</v>
-      </c>
-      <c r="C32" s="3" t="s">
+        <v>40.290088638195</v>
+      </c>
+      <c r="C32" s="4" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B33" s="10" t="n">
+      <c r="B33" s="11" t="n">
         <f aca="false">$B$5/(4*$B$10*$B$12*$B$14)*1000</f>
         <v>71.9178082191781</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="4" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B34" s="11" t="n">
+      <c r="B34" s="12" t="n">
         <f aca="false">$B$17*B22</f>
         <v>22.8571428571429</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="4" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B35" s="11" t="n">
+      <c r="B35" s="12" t="n">
         <f aca="false">$B$17*B23</f>
         <v>42.4590888987174</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="4" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="s">
+      <c r="A36" s="8" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="5" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
+      <c r="A38" s="5" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="5" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="5" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="5" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="5" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2240,198 +2287,198 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="16" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="5" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <f aca="false">SUM(B5:B9)</f>
         <v>20</v>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="3" t="n">
         <f aca="false">SUM(C5:C9)</f>
         <v>42</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="10" t="n">
         <v>800</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="B12" s="17" t="n">
+      <c r="B12" s="18" t="n">
         <f aca="false">B11/(B11+B10)</f>
         <v>0.975609756097561</v>
       </c>
-      <c r="C12" s="17" t="n">
+      <c r="C12" s="18" t="n">
         <f aca="false">B11/(B11+C10)</f>
         <v>0.950118764845606</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="8" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="5" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="5" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="5" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="5" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="5" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="5" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="5" t="s">
         <v>115</v>
       </c>
     </row>
@@ -2452,921 +2499,921 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M27"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="I4" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="J4" s="15" t="s">
+      <c r="J4" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="K4" s="15" t="s">
+      <c r="K4" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="L4" s="15" t="s">
+      <c r="L4" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="M4" s="15" t="s">
+      <c r="M4" s="16" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="G5" s="9" t="n">
+      <c r="G5" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="H5" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="20" t="n">
         <f aca="false">G5*H5</f>
         <v>14</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="L5" s="16" t="s">
+      <c r="L5" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="M5" s="5" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="G6" s="9" t="n">
+      <c r="G6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="18" t="n">
+      <c r="H6" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="I6" s="20" t="n">
         <f aca="false">G6*H6</f>
         <v>12</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="K6" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="L6" s="16" t="s">
+      <c r="L6" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="M6" s="5" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="G7" s="9" t="n">
+      <c r="G7" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="18" t="n">
+      <c r="H7" s="19" t="n">
         <v>0.5</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="I7" s="20" t="n">
         <f aca="false">G7*H7</f>
         <v>0</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="J7" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="K7" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="L7" s="16" t="s">
+      <c r="L7" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M7" s="4" t="s">
+      <c r="M7" s="5" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G8" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="18" t="n">
+      <c r="H8" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="20" t="n">
         <f aca="false">G8*H8</f>
         <v>8</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="J8" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="K8" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="L8" s="16" t="s">
+      <c r="L8" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M8" s="4" t="s">
+      <c r="M8" s="5" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G9" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="18" t="n">
+      <c r="H9" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="20" t="n">
         <f aca="false">G9*H9</f>
         <v>4</v>
       </c>
-      <c r="J9" s="4" t="s">
+      <c r="J9" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="K9" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="L9" s="16" t="s">
+      <c r="L9" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M9" s="4" t="s">
+      <c r="M9" s="5" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="G10" s="9" t="n">
+      <c r="G10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="18" t="n">
+      <c r="H10" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="20" t="n">
         <f aca="false">G10*H10</f>
         <v>15</v>
       </c>
-      <c r="J10" s="4" t="s">
+      <c r="J10" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="K10" s="4" t="s">
+      <c r="K10" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="L10" s="16" t="s">
+      <c r="L10" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="M10" s="4" t="s">
+      <c r="M10" s="5" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="G11" s="9" t="n">
+      <c r="G11" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="18" t="n">
+      <c r="H11" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="I11" s="19" t="n">
+      <c r="I11" s="20" t="n">
         <f aca="false">G11*H11</f>
         <v>25</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="J11" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="K11" s="4" t="s">
+      <c r="K11" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="L11" s="16" t="s">
+      <c r="L11" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="M11" s="4" t="s">
+      <c r="M11" s="5" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="G12" s="9" t="n">
+      <c r="G12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H12" s="18" t="n">
+      <c r="H12" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I12" s="19" t="n">
+      <c r="I12" s="20" t="n">
         <f aca="false">G12*H12</f>
         <v>8</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="J12" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="K12" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="L12" s="16" t="s">
+      <c r="L12" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="M12" s="5" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="G13" s="9" t="n">
+      <c r="G13" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="18" t="n">
+      <c r="H13" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I13" s="19" t="n">
+      <c r="I13" s="20" t="n">
         <f aca="false">G13*H13</f>
         <v>8</v>
       </c>
-      <c r="J13" s="4" t="s">
+      <c r="J13" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="K13" s="4" t="s">
+      <c r="K13" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="L13" s="16" t="s">
+      <c r="L13" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M13" s="4" t="s">
+      <c r="M13" s="5" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="G14" s="9" t="n">
+      <c r="G14" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="18" t="n">
+      <c r="H14" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="I14" s="19" t="n">
+      <c r="I14" s="20" t="n">
         <f aca="false">G14*H14</f>
         <v>5</v>
       </c>
-      <c r="J14" s="4" t="s">
+      <c r="J14" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="K14" s="4" t="s">
+      <c r="K14" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="L14" s="16" t="s">
+      <c r="L14" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M14" s="4" t="s">
+      <c r="M14" s="5" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="G15" s="9" t="n">
+      <c r="G15" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="18" t="n">
+      <c r="H15" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="I15" s="19" t="n">
+      <c r="I15" s="20" t="n">
         <f aca="false">G15*H15</f>
         <v>3</v>
       </c>
-      <c r="J15" s="4" t="s">
+      <c r="J15" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="K15" s="4" t="s">
+      <c r="K15" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="L15" s="16" t="s">
+      <c r="L15" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M15" s="4" t="s">
+      <c r="M15" s="5" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="G16" s="9" t="n">
+      <c r="G16" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H16" s="18" t="n">
+      <c r="H16" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="I16" s="19" t="n">
+      <c r="I16" s="20" t="n">
         <f aca="false">G16*H16</f>
         <v>6</v>
       </c>
-      <c r="J16" s="4" t="s">
+      <c r="J16" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="K16" s="4" t="s">
+      <c r="K16" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="L16" s="16" t="s">
+      <c r="L16" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M16" s="4" t="s">
+      <c r="M16" s="5" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="G17" s="9" t="n">
+      <c r="G17" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H17" s="18" t="n">
+      <c r="H17" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="I17" s="19" t="n">
+      <c r="I17" s="20" t="n">
         <f aca="false">G17*H17</f>
         <v>4</v>
       </c>
-      <c r="J17" s="4" t="s">
+      <c r="J17" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="K17" s="4" t="s">
+      <c r="K17" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="L17" s="16" t="s">
+      <c r="L17" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M17" s="4" t="s">
+      <c r="M17" s="5" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="n">
+      <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="F18" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="G18" s="9" t="n">
+      <c r="G18" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H18" s="18" t="n">
+      <c r="H18" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="I18" s="19" t="n">
+      <c r="I18" s="20" t="n">
         <f aca="false">G18*H18</f>
         <v>3</v>
       </c>
-      <c r="J18" s="4" t="s">
+      <c r="J18" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="K18" s="4" t="s">
+      <c r="K18" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="L18" s="16" t="s">
+      <c r="L18" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M18" s="4"/>
+      <c r="M18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="F19" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="G19" s="9" t="n">
+      <c r="G19" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H19" s="18" t="n">
+      <c r="H19" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="I19" s="19" t="n">
+      <c r="I19" s="20" t="n">
         <f aca="false">G19*H19</f>
         <v>2</v>
       </c>
-      <c r="J19" s="4" t="s">
+      <c r="J19" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="K19" s="4" t="s">
+      <c r="K19" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="L19" s="16" t="s">
+      <c r="L19" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="M19" s="4" t="s">
+      <c r="M19" s="5" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="n">
+      <c r="A20" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="F20" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="G20" s="9" t="n">
+      <c r="G20" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H20" s="18" t="n">
+      <c r="H20" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="I20" s="19" t="n">
+      <c r="I20" s="20" t="n">
         <f aca="false">G20*H20</f>
         <v>2</v>
       </c>
-      <c r="J20" s="4" t="s">
+      <c r="J20" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="K20" s="4" t="s">
+      <c r="K20" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="L20" s="16" t="s">
+      <c r="L20" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="M20" s="4" t="s">
+      <c r="M20" s="5" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="F21" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="G21" s="9" t="n">
+      <c r="G21" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="18" t="n">
+      <c r="H21" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="I21" s="19" t="n">
+      <c r="I21" s="20" t="n">
         <f aca="false">G21*H21</f>
         <v>1</v>
       </c>
-      <c r="J21" s="4" t="s">
+      <c r="J21" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="K21" s="4" t="s">
+      <c r="K21" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="L21" s="16" t="s">
+      <c r="L21" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="M21" s="4" t="s">
+      <c r="M21" s="5" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="n">
+      <c r="A22" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F22" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="G22" s="9" t="n">
+      <c r="G22" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="18" t="n">
+      <c r="H22" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="I22" s="19" t="n">
+      <c r="I22" s="20" t="n">
         <f aca="false">G22*H22</f>
         <v>5</v>
       </c>
-      <c r="J22" s="4" t="s">
+      <c r="J22" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="K22" s="4" t="s">
+      <c r="K22" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="L22" s="16" t="s">
+      <c r="L22" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M22" s="4" t="s">
+      <c r="M22" s="5" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="n">
+      <c r="A23" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F23" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="G23" s="9" t="n">
+      <c r="G23" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="18" t="n">
+      <c r="H23" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="I23" s="19" t="n">
+      <c r="I23" s="20" t="n">
         <f aca="false">G23*H23</f>
         <v>6</v>
       </c>
-      <c r="J23" s="4" t="s">
+      <c r="J23" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="K23" s="4" t="s">
+      <c r="K23" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="L23" s="16" t="s">
+      <c r="L23" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="M23" s="4" t="s">
+      <c r="M23" s="5" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="n">
+      <c r="A24" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="F24" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="G24" s="9" t="n">
+      <c r="G24" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H24" s="18" t="n">
+      <c r="H24" s="19" t="n">
         <v>20</v>
       </c>
-      <c r="I24" s="19" t="n">
+      <c r="I24" s="20" t="n">
         <f aca="false">G24*H24</f>
         <v>20</v>
       </c>
-      <c r="J24" s="4" t="s">
+      <c r="J24" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="K24" s="4" t="s">
+      <c r="K24" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="L24" s="16" t="s">
+      <c r="L24" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="M24" s="4" t="s">
+      <c r="M24" s="5" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H25" s="2" t="s">
+      <c r="H25" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="I25" s="20" t="n">
+      <c r="I25" s="21" t="n">
         <f aca="false">SUM(I5:I24)</f>
         <v>151</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="4" t="s">
         <v>236</v>
       </c>
     </row>
@@ -3387,198 +3434,198 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="B3" s="21" t="n">
+      <c r="B3" s="22" t="n">
         <v>0.79</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="16" t="s">
         <v>240</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="16" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="23" t="n">
         <f aca="false">BOM!I5+BOM!I6</f>
         <v>26</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="23" t="n">
         <f aca="false">SUM(BOM!I8:I11)</f>
         <v>52</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="B8" s="22" t="n">
+      <c r="B8" s="23" t="n">
         <f aca="false">SUM(BOM!I12:I13)</f>
         <v>16</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="23" t="n">
         <f aca="false">SUM(BOM!I14:I21)</f>
         <v>26</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>251</v>
       </c>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="23" t="n">
         <f aca="false">BOM!I22</f>
         <v>5</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B11" s="23" t="n">
         <f aca="false">BOM!I23</f>
         <v>6</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="B12" s="22" t="n">
+      <c r="B12" s="23" t="n">
         <f aca="false">BOM!I24</f>
         <v>20</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="B13" s="20" t="n">
+      <c r="B13" s="21" t="n">
         <f aca="false">SUM(B6:B12)</f>
         <v>151</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="8" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="10" t="n">
         <v>0.75</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="B17" s="9" t="n">
+      <c r="B17" s="10" t="n">
         <v>1.55</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="B18" s="20" t="n">
+      <c r="B18" s="21" t="n">
         <f aca="false">B13*B16</f>
         <v>113.25</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>261</v>
       </c>
-      <c r="B19" s="20" t="n">
+      <c r="B19" s="21" t="n">
         <f aca="false">B13*B17</f>
         <v>234.05</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>262</v>
       </c>
     </row>
@@ -3599,168 +3646,168 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="B3" s="10" t="n">
+      <c r="B3" s="11" t="n">
         <f aca="false">70*280/100</f>
         <v>196</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>266</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="16" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>271</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>273</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>275</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>281</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="3" t="n">
         <f aca="false">SUM(B6:B12)</f>
         <v>160</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="3" t="n">
         <f aca="false">B3-B13</f>
         <v>36</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>284</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>285</v>
       </c>
     </row>
@@ -3781,374 +3828,374 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>287</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="16" t="s">
         <v>288</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="16" t="s">
         <v>240</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="16" t="s">
         <v>289</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="16" t="s">
         <v>290</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="16" t="s">
         <v>292</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="16" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="17" t="s">
         <v>293</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>294</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="E5" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="F5" s="24" t="n">
+      <c r="F5" s="25" t="n">
         <f aca="false">D5*E5</f>
         <v>16</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="5" t="s">
         <v>295</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="H5" s="17" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="17" t="s">
         <v>297</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="D6" s="23" t="n">
+      <c r="D6" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E6" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="F6" s="24" t="n">
+      <c r="F6" s="25" t="n">
         <f aca="false">D6*E6</f>
         <v>16</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="H6" s="16" t="s">
+      <c r="H6" s="17" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="17" t="s">
         <v>301</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="24" t="n">
+      <c r="F7" s="25" t="n">
         <f aca="false">D7*E7</f>
         <v>12</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="5" t="s">
         <v>304</v>
       </c>
-      <c r="H7" s="16" t="s">
+      <c r="H7" s="17" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="17" t="s">
         <v>305</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>306</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>307</v>
       </c>
-      <c r="D8" s="23" t="n">
+      <c r="D8" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="23" t="n">
+      <c r="E8" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="24" t="n">
+      <c r="F8" s="25" t="n">
         <f aca="false">D8*E8</f>
         <v>12</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="5" t="s">
         <v>308</v>
       </c>
-      <c r="H8" s="16" t="s">
+      <c r="H8" s="17" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="17" t="s">
         <v>309</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>311</v>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="23" t="n">
+      <c r="E9" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="24" t="n">
+      <c r="F9" s="25" t="n">
         <f aca="false">D9*E9</f>
         <v>12</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="17" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="17" t="s">
         <v>313</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>314</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>315</v>
       </c>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E10" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="24" t="n">
+      <c r="F10" s="25" t="n">
         <f aca="false">D10*E10</f>
         <v>9</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="5" t="s">
         <v>316</v>
       </c>
-      <c r="H10" s="16" t="s">
+      <c r="H10" s="17" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="17" t="s">
         <v>317</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>319</v>
       </c>
-      <c r="D11" s="23" t="n">
+      <c r="D11" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="23" t="n">
+      <c r="E11" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="24" t="n">
+      <c r="F11" s="25" t="n">
         <f aca="false">D11*E11</f>
         <v>9</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="5" t="s">
         <v>320</v>
       </c>
-      <c r="H11" s="16" t="s">
+      <c r="H11" s="17" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="17" t="s">
         <v>321</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>322</v>
       </c>
-      <c r="D12" s="23" t="n">
+      <c r="D12" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="23" t="n">
+      <c r="E12" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="24" t="n">
+      <c r="F12" s="25" t="n">
         <f aca="false">D12*E12</f>
         <v>9</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="5" t="s">
         <v>323</v>
       </c>
-      <c r="H12" s="16" t="s">
+      <c r="H12" s="17" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="17" t="s">
         <v>324</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="D13" s="23" t="n">
+      <c r="D13" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="23" t="n">
+      <c r="E13" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F13" s="24" t="n">
+      <c r="F13" s="25" t="n">
         <f aca="false">D13*E13</f>
         <v>9</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="5" t="s">
         <v>326</v>
       </c>
-      <c r="H13" s="16" t="s">
+      <c r="H13" s="17" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="17" t="s">
         <v>327</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>328</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="D14" s="23" t="n">
+      <c r="D14" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="23" t="n">
+      <c r="E14" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="24" t="n">
+      <c r="F14" s="25" t="n">
         <f aca="false">D14*E14</f>
         <v>6</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="5" t="s">
         <v>330</v>
       </c>
-      <c r="H14" s="16" t="s">
+      <c r="H14" s="17" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="17" t="s">
         <v>331</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>332</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="D15" s="23" t="n">
+      <c r="D15" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="E15" s="23" t="n">
+      <c r="E15" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="24" t="n">
+      <c r="F15" s="25" t="n">
         <f aca="false">D15*E15</f>
         <v>6</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="5" t="s">
         <v>334</v>
       </c>
-      <c r="H15" s="16" t="s">
+      <c r="H15" s="17" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="17" t="s">
         <v>335</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>336</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="D16" s="23" t="n">
+      <c r="D16" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="23" t="n">
+      <c r="E16" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F16" s="24" t="n">
+      <c r="F16" s="25" t="n">
         <f aca="false">D16*E16</f>
         <v>6</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="5" t="s">
         <v>338</v>
       </c>
-      <c r="H16" s="16" t="s">
+      <c r="H16" s="17" t="s">
         <v>296</v>
       </c>
     </row>
@@ -4169,212 +4216,212 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>339</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="16" t="s">
         <v>340</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="16" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>343</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>344</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>345</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>346</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>347</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>348</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>349</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>351</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>352</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>353</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>354</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>355</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>356</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>357</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>358</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>359</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>360</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>362</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>363</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="5" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>366</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>367</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="5" t="s">
         <v>368</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>369</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="5" t="s">
         <v>233</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Initial kicad schematic draft
</commit_message>
<xml_diff>
--- a/Design Notes/20260609 LibreDAB_planning_pack.xlsx
+++ b/Design Notes/20260609 LibreDAB_planning_pack.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId3"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="373">
   <si>
     <t xml:space="preserve">LibreDAB — Planning Pack (block diagram, BOM, size &amp; risk)</t>
   </si>
@@ -119,10 +119,10 @@
     <t xml:space="preserve">IMPORTANT</t>
   </si>
   <si>
-    <t xml:space="preserve">GaN power devices (EPC23102, LMG2652) are NOT in the LCSC catalogue. They are off-LCSC lines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(Mouser/DigiKey/manufacturer). An all-LCSC HV fallback (Tokmas CID12N65D x4 + drivers) is noted in the BOM.</t>
+    <t xml:space="preserve">GaN power devices (LMG2100R026, LMG2652) are NOT in the LCSC catalogue. They are off-LCSC lines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Mouser/DigiKey/TI) - now an all-TI power stage (single vendor). All-LCSC HV fallback (Tokmas CID12N65D x4 + drivers) noted in BOM.</t>
   </si>
   <si>
     <t xml:space="preserve">DAB Design Calculations (single-phase-shift model)</t>
@@ -308,13 +308,13 @@
     <t xml:space="preserve">Basis / source</t>
   </si>
   <si>
-    <t xml:space="preserve">LV full bridge (2x EPC23102, 6.6 mΩ)</t>
+    <t xml:space="preserve">LV full bridge (2x LMG2100R026, 2.6 mΩ)</t>
   </si>
   <si>
     <t xml:space="preserve">M</t>
   </si>
   <si>
-    <t xml:space="preserve">I_rms^2*Rds + switching; balloons at 35 A low-V corner</t>
+    <t xml:space="preserve">Lower Rds (2.6 mΩ) cuts conduction; 53 A rating eases low-V corner</t>
   </si>
   <si>
     <t xml:space="preserve">HV full bridge (2x LMG2652, 140 mΩ)</t>
@@ -425,22 +425,22 @@
     <t xml:space="preserve">HS+LS GaN half-bridge x2 (full bridge)</t>
   </si>
   <si>
-    <t xml:space="preserve">EPC23102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EPC</t>
+    <t xml:space="preserve">LMG2100R026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TI</t>
   </si>
   <si>
     <t xml:space="preserve">off-LCSC (Mouser/DigiKey)</t>
   </si>
   <si>
-    <t xml:space="preserve">~$5.40/1k; ~$8-9 low qty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://epc-co.com/epc/products/gan-fets-and-ics/epc23102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exposed-top cooling. NOT on LCSC -&gt; self-supply/consign</t>
+    <t xml:space="preserve">~$8-13 low qty; in stock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ti.com/product/LMG2100R026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">93V cont/100V pulsed, 53A, 2.6 mOhm, top-cooled. All-TI w/ HV. NOT on LCSC</t>
   </si>
   <si>
     <t xml:space="preserve">HV bridge</t>
@@ -452,9 +452,6 @@
     <t xml:space="preserve">LMG2652RFBR</t>
   </si>
   <si>
-    <t xml:space="preserve">TI</t>
-  </si>
-  <si>
     <t xml:space="preserve">~$7-8; 12-wk lead</t>
   </si>
   <si>
@@ -761,7 +758,7 @@
     <t xml:space="preserve">Semiconductors (GaN)</t>
   </si>
   <si>
-    <t xml:space="preserve">EPC23102 x2 + LMG2652 x2; off-LCSC</t>
+    <t xml:space="preserve">LMG2100R026 x2 + LMG2652 x2; all-TI, off-LCSC</t>
   </si>
   <si>
     <t xml:space="preserve">Magnetics (custom, UK)</t>
@@ -836,7 +833,7 @@
     <t xml:space="preserve">LV full bridge + input caps</t>
   </si>
   <si>
-    <t xml:space="preserve">2x EPC23102 (3.5x5 mm) + decoupling + heavy-copper pour</t>
+    <t xml:space="preserve">2x LMG2100R026 (7x4.5 mm) + decoupling + heavy-copper pour</t>
   </si>
   <si>
     <t xml:space="preserve">HV full bridge + bus caps</t>
@@ -926,10 +923,10 @@
     <t xml:space="preserve">Thermal/Device</t>
   </si>
   <si>
-    <t xml:space="preserve">LV switch at 23.8 V full-power corner ~35 A vs 35 A rating -&gt; marginal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Derate power at low SoC; conduction+top heatsink cooling; consider paralleling / 2 oz copper</t>
+    <t xml:space="preserve">LV switch current at 23.8 V full-power corner (~42 A) vs 53 A rating -&gt; comfortable margin; thermal still to manage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Top-side heatsink + conduction; verify 1 MHz thermal derating at worst corner</t>
   </si>
   <si>
     <t xml:space="preserve">S-01</t>
@@ -1055,19 +1052,28 @@
     <t xml:space="preserve">URL</t>
   </si>
   <si>
-    <t xml:space="preserve">EPC23102 product page / datasheet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LV GaN: 100 V, 35 A, 6.6 mΩ, exposed-top cooling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EPC23102 launch (Semiconductor Today)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">96% peak eff @1 MHz, $5.40/1k, 3.5x5 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://semiconductor-today.com/news_items/2022/aug/epc-100822.shtml</t>
+    <t xml:space="preserve">TI LMG2100R026 product page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LV GaN: 93 V cont/100 V pulsed, 53 A, 2.6 mΩ, integrated driver, top-cooled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TI LMG2100R026 datasheet (PDF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electrical specs, 7.0x4.5 mm 18-VQFN, UVLO/clamp protection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ti.com/lit/ds/symlink/lmg2100r026.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DigiKey LMG2100R026VBNR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Availability (in stock) &amp; low-qty pricing - verify before order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/en/products/detail/texas-instruments/LMG2100R026VBNR/25811484</t>
   </si>
   <si>
     <t xml:space="preserve">TI LMG2652 product page</t>
@@ -1146,7 +1152,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0"/>
@@ -1155,6 +1161,7 @@
     <numFmt numFmtId="169" formatCode="0.0%"/>
     <numFmt numFmtId="170" formatCode="\£#,##0.00"/>
     <numFmt numFmtId="171" formatCode="0.00"/>
+    <numFmt numFmtId="172" formatCode="General"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -1298,108 +1305,104 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="170" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="172" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1473,49 +1476,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>409320</xdr:colOff>
-      <xdr:row>54</xdr:row>
-      <xdr:rowOff>117000</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 1"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="5133240"/>
-          <a:ext cx="11054520" cy="5451120"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1699,159 +1659,159 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B22"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="105"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="105"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4"/>
-      <c r="B3" s="5"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4"/>
-      <c r="B7" s="5"/>
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6"/>
-      <c r="B11" s="5"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="5"/>
+      <c r="B12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4"/>
-      <c r="B20" s="5"/>
+      <c r="A20" s="3"/>
+      <c r="B20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4"/>
-      <c r="B22" s="5" t="s">
+      <c r="A22" s="3"/>
+      <c r="B22" s="4" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1863,7 +1823,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1873,400 +1832,400 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C42"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="8" t="n">
         <v>42</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="9" t="n">
         <v>23.8</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="9" t="n">
         <v>58.8</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="9" t="n">
         <v>400</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="9" t="n">
         <v>800</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="9" t="n">
         <v>1000000</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="10" t="n">
-        <v>17</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="B11" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="9" t="n">
         <v>3.7E-006</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="3" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="9" t="n">
         <v>0.000146</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="3" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="3" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="9" t="n">
         <v>0.95</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="9" t="n">
         <v>1.2</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="7" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B20" s="11" t="n">
+      <c r="B20" s="10" t="n">
         <f aca="false">$B$11*$B$12</f>
-        <v>17</v>
-      </c>
-      <c r="C20" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="12" t="n">
+      <c r="B21" s="11" t="n">
         <f aca="false">$B$8/$B$11</f>
-        <v>23.5294117647059</v>
-      </c>
-      <c r="C21" s="4" t="s">
+        <v>36.3636363636364</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B22" s="12" t="n">
+      <c r="B22" s="11" t="n">
         <f aca="false">$B$9/$B$5</f>
         <v>19.047619047619</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="3" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="12" t="n">
+      <c r="B23" s="11" t="n">
         <f aca="false">$B$9/($B$16*$B$6)</f>
         <v>35.3825740822645</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="3" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="13" t="n">
+      <c r="B24" s="12" t="n">
         <f aca="false">$B$15*PI()/180</f>
         <v>0.872664625997165</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="3" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B25" s="13" t="n">
+      <c r="B25" s="12" t="n">
         <f aca="false">B24*(1-B24/PI())</f>
         <v>0.630257785442397</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B26" s="14" t="n">
+      <c r="B26" s="13" t="n">
         <f aca="false">$B$5*B21*B25/(2*PI()*$B$10*$B$9)</f>
-        <v>1.23910675381264E-007</v>
-      </c>
-      <c r="C26" s="4" t="s">
+        <v>1.91498316498317E-007</v>
+      </c>
+      <c r="C26" s="3" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B27" s="11" t="n">
+      <c r="B27" s="10" t="n">
         <f aca="false">B26*1000000000</f>
-        <v>123.910675381264</v>
-      </c>
-      <c r="C27" s="4" t="s">
+        <v>191.498316498317</v>
+      </c>
+      <c r="C27" s="3" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B28" s="12" t="n">
+      <c r="B28" s="11" t="n">
         <f aca="false">B26*$B$11^2*1000000</f>
-        <v>35.8101851851852</v>
-      </c>
-      <c r="C28" s="4" t="s">
+        <v>23.1712962962963</v>
+      </c>
+      <c r="C28" s="3" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B29" s="14" t="n">
+      <c r="B29" s="13" t="n">
         <f aca="false">$B$13*$B$12^2</f>
         <v>3.7E-006</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="3" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B30" s="15" t="n">
+      <c r="B30" s="14" t="n">
         <f aca="false">B26/B29</f>
-        <v>0.0334893717246659</v>
-      </c>
-      <c r="C30" s="4" t="s">
+        <v>0.0517563017563018</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B31" s="13" t="n">
+      <c r="B31" s="12" t="n">
         <f aca="false">$B$8/(4*$B$10*B20*$B$14)</f>
-        <v>0.040290088638195</v>
-      </c>
-      <c r="C31" s="4" t="s">
+        <v>0.062266500622665</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B32" s="11" t="n">
+      <c r="B32" s="10" t="n">
         <f aca="false">B31*1000</f>
-        <v>40.290088638195</v>
-      </c>
-      <c r="C32" s="4" t="s">
+        <v>62.266500622665</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B33" s="11" t="n">
+      <c r="B33" s="10" t="n">
         <f aca="false">$B$5/(4*$B$10*$B$12*$B$14)*1000</f>
         <v>71.9178082191781</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="3" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B34" s="12" t="n">
+      <c r="B34" s="11" t="n">
         <f aca="false">$B$17*B22</f>
         <v>22.8571428571429</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="3" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B35" s="12" t="n">
+      <c r="B35" s="11" t="n">
         <f aca="false">$B$17*B23</f>
         <v>42.4590888987174</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="3" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="8" t="s">
+      <c r="A36" s="7" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="s">
+      <c r="A37" s="4" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="4" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5" t="s">
+      <c r="A39" s="4" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="4" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5" t="s">
+      <c r="A41" s="4" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="4" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2287,198 +2246,198 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="15" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="C5" s="10" t="n">
-        <v>22</v>
-      </c>
-      <c r="D5" s="17" t="s">
+      <c r="D6" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B6" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="D6" s="17" t="s">
+      <c r="E6" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B7" s="10" t="n">
+      <c r="E7" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="C7" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B8" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="B9" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="4" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="2" t="n">
         <f aca="false">SUM(B5:B9)</f>
-        <v>20</v>
-      </c>
-      <c r="C10" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C10" s="2" t="n">
         <f aca="false">SUM(C5:C9)</f>
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="9" t="n">
         <v>800</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="17" t="n">
         <f aca="false">B11/(B11+B10)</f>
-        <v>0.975609756097561</v>
-      </c>
-      <c r="C12" s="18" t="n">
+        <v>0.97799511002445</v>
+      </c>
+      <c r="C12" s="17" t="n">
         <f aca="false">B11/(B11+C10)</f>
-        <v>0.950118764845606</v>
+        <v>0.962695547533093</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="4" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="4" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="4" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="4" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="4" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="4" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="4" t="s">
         <v>115</v>
       </c>
     </row>
@@ -2499,922 +2458,922 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M27"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="J4" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="K4" s="16" t="s">
+      <c r="K4" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="L4" s="16" t="s">
+      <c r="L4" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="M4" s="16" t="s">
+      <c r="M4" s="15" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="G5" s="10" t="n">
+      <c r="G5" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="19" t="n">
-        <v>7</v>
-      </c>
-      <c r="I5" s="20" t="n">
+      <c r="H5" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="I5" s="19" t="n">
         <f aca="false">G5*H5</f>
-        <v>14</v>
-      </c>
-      <c r="J5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="K5" s="5" t="s">
+      <c r="K5" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="L5" s="17" t="s">
+      <c r="L5" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="M5" s="5" t="s">
+      <c r="M5" s="4" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="F6" s="4" t="s">
+      <c r="E6" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="G6" s="10" t="n">
+      <c r="G6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="19" t="n">
+      <c r="H6" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="I6" s="20" t="n">
+      <c r="I6" s="19" t="n">
         <f aca="false">G6*H6</f>
         <v>12</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="J6" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="K6" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="L6" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="M6" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="L6" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="M6" s="5" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="D7" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="19" t="n">
+      <c r="H7" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="I7" s="20" t="n">
+      <c r="I7" s="19" t="n">
         <f aca="false">G7*H7</f>
         <v>0</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="J7" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="K7" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="L7" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="M7" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="L7" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="M7" s="5" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="G8" s="10" t="n">
+      <c r="G8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="19" t="n">
+      <c r="H8" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="I8" s="20" t="n">
+      <c r="I8" s="19" t="n">
         <f aca="false">G8*H8</f>
         <v>8</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="J8" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="K8" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="K8" s="5" t="s">
+      <c r="L8" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="M8" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="L8" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="M8" s="5" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="G9" s="10" t="n">
+      <c r="G9" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="19" t="n">
+      <c r="H9" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="I9" s="20" t="n">
+      <c r="I9" s="19" t="n">
         <f aca="false">G9*H9</f>
         <v>4</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="J9" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="K9" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="L9" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="M9" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="L9" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="M9" s="5" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="E10" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="G10" s="10" t="n">
+      <c r="F10" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="19" t="n">
+      <c r="H10" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="I10" s="20" t="n">
+      <c r="I10" s="19" t="n">
         <f aca="false">G10*H10</f>
         <v>15</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="J10" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="K10" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="K10" s="5" t="s">
+      <c r="L10" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="M10" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="L10" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="M10" s="5" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="E11" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="G11" s="10" t="n">
+      <c r="F11" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G11" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="19" t="n">
+      <c r="H11" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="I11" s="20" t="n">
+      <c r="I11" s="19" t="n">
         <f aca="false">G11*H11</f>
         <v>25</v>
       </c>
-      <c r="J11" s="5" t="s">
+      <c r="J11" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="L11" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="M11" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="K11" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="L11" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="M11" s="5" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="n">
+      <c r="C12" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="G12" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="I12" s="20" t="n">
+      <c r="I12" s="19" t="n">
         <f aca="false">G12*H12</f>
         <v>8</v>
       </c>
-      <c r="J12" s="5" t="s">
+      <c r="J12" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="K12" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="K12" s="5" t="s">
+      <c r="L12" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="M12" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="L12" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="M12" s="5" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="4" t="s">
+      <c r="C13" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="F13" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="G13" s="10" t="n">
+      <c r="G13" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="19" t="n">
+      <c r="H13" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="I13" s="20" t="n">
+      <c r="I13" s="19" t="n">
         <f aca="false">G13*H13</f>
         <v>8</v>
       </c>
-      <c r="J13" s="5" t="s">
+      <c r="J13" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="K13" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="K13" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="L13" s="17" t="s">
+      <c r="L13" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="M13" s="5" t="s">
+      <c r="M13" s="4" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="G14" s="10" t="n">
+      <c r="G14" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="19" t="n">
+      <c r="H14" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="I14" s="20" t="n">
+      <c r="I14" s="19" t="n">
         <f aca="false">G14*H14</f>
         <v>5</v>
       </c>
-      <c r="J14" s="5" t="s">
+      <c r="J14" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="K14" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="K14" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="L14" s="17" t="s">
+      <c r="L14" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="M14" s="5" t="s">
+      <c r="M14" s="4" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="F15" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="G15" s="10" t="n">
+      <c r="G15" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="19" t="n">
+      <c r="H15" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="I15" s="20" t="n">
+      <c r="I15" s="19" t="n">
         <f aca="false">G15*H15</f>
         <v>3</v>
       </c>
-      <c r="J15" s="5" t="s">
+      <c r="J15" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="K15" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="K15" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="L15" s="17" t="s">
+      <c r="L15" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="M15" s="5" t="s">
+      <c r="M15" s="4" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="4" t="s">
+      <c r="C16" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="F16" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="G16" s="10" t="n">
+      <c r="G16" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H16" s="19" t="n">
+      <c r="H16" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="I16" s="20" t="n">
+      <c r="I16" s="19" t="n">
         <f aca="false">G16*H16</f>
         <v>6</v>
       </c>
-      <c r="J16" s="5" t="s">
+      <c r="J16" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="K16" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="K16" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="L16" s="17" t="s">
+      <c r="L16" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="M16" s="5" t="s">
+      <c r="M16" s="4" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="4" t="s">
+      <c r="C17" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="F17" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="G17" s="10" t="n">
+      <c r="G17" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H17" s="19" t="n">
+      <c r="H17" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="I17" s="20" t="n">
+      <c r="I17" s="19" t="n">
         <f aca="false">G17*H17</f>
         <v>4</v>
       </c>
-      <c r="J17" s="5" t="s">
+      <c r="J17" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="K17" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="K17" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="L17" s="17" t="s">
+      <c r="L17" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="M17" s="5" t="s">
+      <c r="M17" s="4" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="F18" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="G18" s="10" t="n">
+      <c r="G18" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H18" s="19" t="n">
+      <c r="H18" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="I18" s="20" t="n">
+      <c r="I18" s="19" t="n">
         <f aca="false">G18*H18</f>
         <v>3</v>
       </c>
-      <c r="J18" s="5" t="s">
+      <c r="J18" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="K18" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="K18" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="L18" s="17" t="s">
+      <c r="L18" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="M18" s="5"/>
+      <c r="M18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="n">
+      <c r="A19" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="C19" s="5" t="s">
+      <c r="B19" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="F19" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="G19" s="10" t="n">
+      <c r="G19" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H19" s="19" t="n">
+      <c r="H19" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="I19" s="20" t="n">
+      <c r="I19" s="19" t="n">
         <f aca="false">G19*H19</f>
         <v>2</v>
       </c>
-      <c r="J19" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="K19" s="5" t="s">
+      <c r="J19" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="M19" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="L19" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="M19" s="5" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="D20" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F20" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="F20" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="G20" s="10" t="n">
+      <c r="G20" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H20" s="19" t="n">
+      <c r="H20" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="I20" s="20" t="n">
+      <c r="I20" s="19" t="n">
         <f aca="false">G20*H20</f>
         <v>2</v>
       </c>
-      <c r="J20" s="5" t="s">
+      <c r="J20" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="K20" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="K20" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="L20" s="17" t="s">
+      <c r="L20" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="M20" s="5" t="s">
+      <c r="M20" s="4" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="4" t="s">
+      <c r="C21" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F21" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="F21" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="G21" s="10" t="n">
+      <c r="G21" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="19" t="n">
+      <c r="H21" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="I21" s="20" t="n">
+      <c r="I21" s="19" t="n">
         <f aca="false">G21*H21</f>
         <v>1</v>
       </c>
-      <c r="J21" s="5" t="s">
+      <c r="J21" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="K21" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="K21" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="L21" s="17" t="s">
+      <c r="L21" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="M21" s="5" t="s">
+      <c r="M21" s="4" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="4" t="s">
+      <c r="C22" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="D22" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F22" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="F22" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="G22" s="10" t="n">
+      <c r="G22" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="19" t="n">
+      <c r="H22" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="I22" s="20" t="n">
+      <c r="I22" s="19" t="n">
         <f aca="false">G22*H22</f>
         <v>5</v>
       </c>
-      <c r="J22" s="5" t="s">
+      <c r="J22" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="K22" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="K22" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="L22" s="17" t="s">
+      <c r="L22" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="M22" s="5" t="s">
+      <c r="M22" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="4" t="s">
+      <c r="C23" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="D23" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="E23" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F23" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="E23" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="G23" s="10" t="n">
+      <c r="G23" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="19" t="n">
+      <c r="H23" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="I23" s="20" t="n">
+      <c r="I23" s="19" t="n">
         <f aca="false">G23*H23</f>
         <v>6</v>
       </c>
-      <c r="J23" s="5" t="s">
+      <c r="J23" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="M23" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="K23" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="L23" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="M23" s="5" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="n">
+      <c r="C24" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="G24" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="19" t="n">
-        <v>20</v>
-      </c>
-      <c r="I24" s="20" t="n">
+      <c r="I24" s="19" t="n">
         <f aca="false">G24*H24</f>
         <v>20</v>
       </c>
-      <c r="J24" s="5" t="s">
+      <c r="J24" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="K24" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="K24" s="5" t="s">
+      <c r="L24" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="M24" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="L24" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="M24" s="5" t="s">
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H25" s="2" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H25" s="3" t="s">
+      <c r="I25" s="20" t="n">
+        <f aca="false">SUM(I5:I24)</f>
+        <v>153</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="3" t="s">
         <v>235</v>
-      </c>
-      <c r="I25" s="21" t="n">
-        <f aca="false">SUM(I5:I24)</f>
-        <v>151</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="4" t="s">
-        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -3434,199 +3393,199 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="B3" s="21" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="B3" s="22" t="n">
-        <v>0.79</v>
-      </c>
-      <c r="C3" s="4" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="15" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="s">
+      <c r="B5" s="15" t="s">
         <v>240</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="C5" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5" s="15" t="s">
         <v>241</v>
       </c>
-      <c r="C5" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="D5" s="16" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="B6" s="22" t="n">
+        <f aca="false">BOM!I5+BOM!I6</f>
+        <v>28</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="B6" s="23" t="n">
-        <f aca="false">BOM!I5+BOM!I6</f>
-        <v>26</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="D6" s="5" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="B7" s="23" t="n">
+      <c r="B7" s="22" t="n">
         <f aca="false">SUM(BOM!I8:I11)</f>
         <v>52</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="4" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="B8" s="23" t="n">
+      <c r="B8" s="22" t="n">
         <f aca="false">SUM(BOM!I12:I13)</f>
         <v>16</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="B9" s="23" t="n">
+      <c r="B9" s="22" t="n">
         <f aca="false">SUM(BOM!I14:I21)</f>
         <v>26</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="4" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>251</v>
-      </c>
-      <c r="B10" s="23" t="n">
+      <c r="B10" s="22" t="n">
         <f aca="false">BOM!I22</f>
         <v>5</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>252</v>
+      <c r="D10" s="4" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="B11" s="23" t="n">
+      <c r="A11" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="B11" s="22" t="n">
         <f aca="false">BOM!I23</f>
         <v>6</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="4" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="B12" s="23" t="n">
+      <c r="B12" s="22" t="n">
         <f aca="false">BOM!I24</f>
         <v>20</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="B13" s="20" t="n">
+        <f aca="false">SUM(B6:B12)</f>
+        <v>153</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="B13" s="21" t="n">
-        <f aca="false">SUM(B6:B12)</f>
-        <v>151</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="B16" s="9" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="B16" s="10" t="n">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="B17" s="9" t="n">
+        <v>1.55</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="B17" s="10" t="n">
-        <v>1.55</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="B18" s="20" t="n">
+        <f aca="false">B13*B16</f>
+        <v>114.75</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="B18" s="21" t="n">
-        <f aca="false">B13*B16</f>
-        <v>113.25</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="B19" s="20" t="n">
+        <f aca="false">B13*B17</f>
+        <v>237.15</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
         <v>261</v>
-      </c>
-      <c r="B19" s="21" t="n">
-        <f aca="false">B13*B17</f>
-        <v>234.05</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
-        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -3646,169 +3605,169 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="B3" s="11" t="n">
+      <c r="B3" s="10" t="n">
         <f aca="false">70*280/100</f>
         <v>196</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="15" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="B5" s="16" t="s">
+      <c r="C5" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="D5" s="15" t="s">
         <v>266</v>
       </c>
-      <c r="C5" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="D5" s="16" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="B6" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="B6" s="10" t="n">
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="B7" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C7" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="B7" s="10" t="n">
-        <v>22</v>
-      </c>
-      <c r="C7" s="17" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="C8" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="B8" s="10" t="n">
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="B10" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C10" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="B9" s="10" t="n">
-        <v>25</v>
-      </c>
-      <c r="C9" s="17" t="s">
+      <c r="D10" s="4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C11" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>276</v>
-      </c>
-      <c r="B10" s="10" t="n">
-        <v>18</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="B11" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="D11" s="5" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="B12" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="B12" s="10" t="n">
-        <v>35</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="D12" s="5" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" s="2" t="n">
         <f aca="false">SUM(B6:B12)</f>
         <v>160</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="B14" s="3" t="n">
+      <c r="A14" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B14" s="2" t="n">
         <f aca="false">B3-B13</f>
         <v>36</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>284</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>285</v>
       </c>
     </row>
   </sheetData>
@@ -3828,375 +3787,375 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
+      <c r="B4" s="15" t="s">
+        <v>239</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>288</v>
       </c>
-      <c r="B4" s="16" t="s">
-        <v>240</v>
-      </c>
-      <c r="C4" s="16" t="s">
+      <c r="D4" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="E4" s="15" t="s">
         <v>289</v>
       </c>
-      <c r="D4" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="E4" s="16" t="s">
+      <c r="F4" s="15" t="s">
         <v>290</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="G4" s="15" t="s">
         <v>291</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="H4" s="15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16" t="s">
         <v>292</v>
       </c>
-      <c r="H4" s="16" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="s">
+      <c r="B5" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>293</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>294</v>
-      </c>
-      <c r="D5" s="24" t="n">
+      <c r="D5" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="24" t="n">
+      <c r="E5" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="F5" s="25" t="n">
+      <c r="F5" s="24" t="n">
         <f aca="false">D5*E5</f>
         <v>16</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="H5" s="16" t="s">
         <v>295</v>
       </c>
-      <c r="H5" s="17" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="s">
+      <c r="B6" s="4" t="s">
         <v>297</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>298</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="24" t="n">
+        <f aca="false">D6*E6</f>
+        <v>6</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>299</v>
       </c>
-      <c r="D6" s="24" t="n">
+      <c r="H6" s="16" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>300</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="D7" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="24" t="n">
-        <v>4</v>
-      </c>
-      <c r="F6" s="25" t="n">
-        <f aca="false">D6*E6</f>
-        <v>16</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>300</v>
-      </c>
-      <c r="H6" s="17" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
-        <v>301</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>302</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>303</v>
-      </c>
-      <c r="D7" s="24" t="n">
-        <v>4</v>
-      </c>
-      <c r="E7" s="24" t="n">
+      <c r="E7" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="25" t="n">
+      <c r="F7" s="24" t="n">
         <f aca="false">D7*E7</f>
         <v>12</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
         <v>304</v>
       </c>
-      <c r="H7" s="17" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
+      <c r="B8" s="4" t="s">
         <v>305</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>306</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>307</v>
-      </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="24" t="n">
+      <c r="E8" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="25" t="n">
+      <c r="F8" s="24" t="n">
         <f aca="false">D8*E8</f>
         <v>12</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
         <v>308</v>
       </c>
-      <c r="H8" s="17" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
+      <c r="B9" s="4" t="s">
         <v>309</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>310</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>311</v>
-      </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="E9" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="25" t="n">
+      <c r="F9" s="24" t="n">
         <f aca="false">D9*E9</f>
         <v>12</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="H9" s="16" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="16" t="s">
         <v>312</v>
       </c>
-      <c r="H9" s="17" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
+      <c r="B10" s="4" t="s">
         <v>313</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="4" t="s">
         <v>314</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>315</v>
-      </c>
-      <c r="D10" s="24" t="n">
+      <c r="D10" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="24" t="n">
+      <c r="E10" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="25" t="n">
+      <c r="F10" s="24" t="n">
         <f aca="false">D10*E10</f>
         <v>9</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="H10" s="16" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="16" t="s">
         <v>316</v>
       </c>
-      <c r="H10" s="17" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
+      <c r="B11" s="4" t="s">
         <v>317</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="C11" s="4" t="s">
         <v>318</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>319</v>
-      </c>
-      <c r="D11" s="24" t="n">
+      <c r="D11" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="24" t="n">
+      <c r="E11" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="25" t="n">
+      <c r="F11" s="24" t="n">
         <f aca="false">D11*E11</f>
         <v>9</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="G11" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="H11" s="16" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="16" t="s">
         <v>320</v>
       </c>
-      <c r="H11" s="17" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
+      <c r="B12" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>322</v>
-      </c>
-      <c r="D12" s="24" t="n">
+      <c r="D12" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="24" t="n">
+      <c r="E12" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="25" t="n">
+      <c r="F12" s="24" t="n">
         <f aca="false">D12*E12</f>
         <v>9</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="H12" s="16" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="16" t="s">
         <v>323</v>
       </c>
-      <c r="H12" s="17" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17" t="s">
+      <c r="B13" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>324</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="D13" s="24" t="n">
+      <c r="D13" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="24" t="n">
+      <c r="E13" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F13" s="25" t="n">
+      <c r="F13" s="24" t="n">
         <f aca="false">D13*E13</f>
         <v>9</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="H13" s="16" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="16" t="s">
         <v>326</v>
       </c>
-      <c r="H13" s="17" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="s">
+      <c r="B14" s="4" t="s">
         <v>327</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="4" t="s">
         <v>328</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="D14" s="24" t="n">
+      <c r="D14" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="24" t="n">
+      <c r="E14" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="25" t="n">
+      <c r="F14" s="24" t="n">
         <f aca="false">D14*E14</f>
         <v>6</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="G14" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="H14" s="16" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="s">
         <v>330</v>
       </c>
-      <c r="H14" s="17" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="s">
+      <c r="B15" s="4" t="s">
         <v>331</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="4" t="s">
         <v>332</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>333</v>
-      </c>
-      <c r="D15" s="24" t="n">
+      <c r="D15" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="E15" s="24" t="n">
+      <c r="E15" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="25" t="n">
+      <c r="F15" s="24" t="n">
         <f aca="false">D15*E15</f>
         <v>6</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="G15" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="H15" s="16" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="s">
         <v>334</v>
       </c>
-      <c r="H15" s="17" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="s">
+      <c r="B16" s="4" t="s">
         <v>335</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="4" t="s">
         <v>336</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>337</v>
-      </c>
-      <c r="D16" s="24" t="n">
+      <c r="D16" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="24" t="n">
+      <c r="E16" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F16" s="25" t="n">
+      <c r="F16" s="24" t="n">
         <f aca="false">D16*E16</f>
         <v>6</v>
       </c>
-      <c r="G16" s="5" t="s">
-        <v>338</v>
-      </c>
-      <c r="H16" s="17" t="s">
-        <v>296</v>
+      <c r="G16" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="H16" s="16" t="s">
+        <v>295</v>
       </c>
     </row>
   </sheetData>
@@ -4215,214 +4174,228 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="C3" s="15" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="16" t="s">
-        <v>118</v>
-      </c>
-      <c r="B3" s="16" t="s">
-        <v>122</v>
-      </c>
-      <c r="C3" s="16" t="s">
+      <c r="D3" s="15" t="s">
         <v>340</v>
       </c>
-      <c r="D3" s="16" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>342</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="4" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>343</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>344</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>345</v>
       </c>
-      <c r="D5" s="5" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>347</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="4" t="s">
         <v>348</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>143</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>349</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>350</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>352</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>151</v>
-      </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>354</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>355</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>356</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>358</v>
-      </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="4" t="s">
         <v>359</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>165</v>
-      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="C12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>360</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="n">
+      <c r="C12" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>361</v>
-      </c>
-      <c r="C13" s="5" t="s">
+      <c r="B13" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>362</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>209</v>
+      <c r="D13" s="4" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>363</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="4" t="s">
         <v>364</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="4" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="4" t="s">
         <v>367</v>
       </c>
-      <c r="D15" s="5" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>233</v>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Schematic updates still setting up
</commit_message>
<xml_diff>
--- a/Design Notes/20260609 LibreDAB_planning_pack.xlsx
+++ b/Design Notes/20260609 LibreDAB_planning_pack.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId3"/>
@@ -482,7 +482,7 @@
     <t xml:space="preserve">https://www.lcsc.com/product-detail/C21547657.html</t>
   </si>
   <si>
-    <t xml:space="preserve">Alternative path: needs 4x isolated gate driver+bias (more parts)</t>
+    <t xml:space="preserve">Alternative path: needs 4 x modules instead of 2 x</t>
   </si>
   <si>
     <t xml:space="preserve">Magnetics</t>
@@ -1152,7 +1152,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0"/>
@@ -1161,7 +1161,6 @@
     <numFmt numFmtId="169" formatCode="0.0%"/>
     <numFmt numFmtId="170" formatCode="\£#,##0.00"/>
     <numFmt numFmtId="171" formatCode="0.00"/>
-    <numFmt numFmtId="172" formatCode="General"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -1305,104 +1304,108 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1659,159 +1662,159 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B22"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="105"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="105"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="4"/>
+      <c r="B3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
+      <c r="A7" s="4"/>
+      <c r="B7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
-      <c r="B11" s="4"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="4"/>
+      <c r="B12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3"/>
-      <c r="B20" s="4"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3"/>
-      <c r="B22" s="4" t="s">
+      <c r="A22" s="4"/>
+      <c r="B22" s="5" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1832,400 +1835,400 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C42"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="8" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="9" t="n">
         <v>42</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="10" t="n">
         <v>23.8</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="10" t="n">
         <v>58.8</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="10" t="n">
         <v>400</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="10" t="n">
         <v>800</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="10" t="n">
         <v>3.7E-006</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="10" t="n">
         <v>0.000146</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="10" t="n">
         <v>0.95</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="9" t="n">
+      <c r="B17" s="10" t="n">
         <v>1.2</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="8" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="11" t="n">
         <f aca="false">$B$11*$B$12</f>
         <v>11</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B21" s="12" t="n">
         <f aca="false">$B$8/$B$11</f>
         <v>36.3636363636364</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="4" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B22" s="11" t="n">
+      <c r="B22" s="12" t="n">
         <f aca="false">$B$9/$B$5</f>
         <v>19.047619047619</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="4" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="11" t="n">
+      <c r="B23" s="12" t="n">
         <f aca="false">$B$9/($B$16*$B$6)</f>
         <v>35.3825740822645</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="4" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="12" t="n">
+      <c r="B24" s="13" t="n">
         <f aca="false">$B$15*PI()/180</f>
         <v>0.872664625997165</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="4" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B25" s="12" t="n">
+      <c r="B25" s="13" t="n">
         <f aca="false">B24*(1-B24/PI())</f>
         <v>0.630257785442397</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B26" s="13" t="n">
+      <c r="B26" s="14" t="n">
         <f aca="false">$B$5*B21*B25/(2*PI()*$B$10*$B$9)</f>
         <v>1.91498316498317E-007</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="4" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B27" s="10" t="n">
+      <c r="B27" s="11" t="n">
         <f aca="false">B26*1000000000</f>
         <v>191.498316498317</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="4" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B28" s="11" t="n">
+      <c r="B28" s="12" t="n">
         <f aca="false">B26*$B$11^2*1000000</f>
         <v>23.1712962962963</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="4" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
+      <c r="A29" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B29" s="13" t="n">
+      <c r="B29" s="14" t="n">
         <f aca="false">$B$13*$B$12^2</f>
         <v>3.7E-006</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="4" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B30" s="14" t="n">
+      <c r="B30" s="15" t="n">
         <f aca="false">B26/B29</f>
         <v>0.0517563017563018</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="4" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B31" s="12" t="n">
+      <c r="B31" s="13" t="n">
         <f aca="false">$B$8/(4*$B$10*B20*$B$14)</f>
         <v>0.062266500622665</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="11" t="n">
         <f aca="false">B31*1000</f>
         <v>62.266500622665</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="4" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B33" s="10" t="n">
+      <c r="B33" s="11" t="n">
         <f aca="false">$B$5/(4*$B$10*$B$12*$B$14)*1000</f>
         <v>71.9178082191781</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="4" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B34" s="11" t="n">
+      <c r="B34" s="12" t="n">
         <f aca="false">$B$17*B22</f>
         <v>22.8571428571429</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="4" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B35" s="11" t="n">
+      <c r="B35" s="12" t="n">
         <f aca="false">$B$17*B23</f>
         <v>42.4590888987174</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="4" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="s">
+      <c r="A36" s="8" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="5" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
+      <c r="A38" s="5" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="5" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="5" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="5" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="5" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2246,198 +2249,198 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="16" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="5" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <f aca="false">SUM(B5:B9)</f>
         <v>18</v>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="3" t="n">
         <f aca="false">SUM(C5:C9)</f>
         <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="10" t="n">
         <v>800</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="B12" s="17" t="n">
+      <c r="B12" s="18" t="n">
         <f aca="false">B11/(B11+B10)</f>
         <v>0.97799511002445</v>
       </c>
-      <c r="C12" s="17" t="n">
+      <c r="C12" s="18" t="n">
         <f aca="false">B11/(B11+C10)</f>
         <v>0.962695547533093</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="8" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="5" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="5" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="5" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="5" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="5" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="5" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="5" t="s">
         <v>115</v>
       </c>
     </row>
@@ -2458,921 +2461,922 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M27"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="25.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="16" t="s">
         <v>121</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="I4" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="J4" s="15" t="s">
+      <c r="J4" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="K4" s="15" t="s">
+      <c r="K4" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="L4" s="15" t="s">
+      <c r="L4" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="M4" s="15" t="s">
+      <c r="M4" s="16" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="G5" s="9" t="n">
+      <c r="G5" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="H5" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="20" t="n">
         <f aca="false">G5*H5</f>
         <v>16</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="L5" s="16" t="s">
+      <c r="L5" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="M5" s="5" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="G6" s="9" t="n">
+      <c r="G6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="I6" s="20" t="n">
+        <f aca="false">G6*H6</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="L6" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" s="19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I7" s="20" t="n">
+        <f aca="false">G7*H7</f>
         <v>2</v>
       </c>
-      <c r="H6" s="18" t="n">
-        <v>6</v>
-      </c>
-      <c r="I6" s="19" t="n">
-        <f aca="false">G6*H6</f>
-        <v>12</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="L6" s="16" t="s">
+      <c r="J7" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="L7" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M6" s="4" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="G7" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="18" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="I7" s="19" t="n">
-        <f aca="false">G7*H7</f>
-        <v>0</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="L7" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="M7" s="4" t="s">
+      <c r="M7" s="5" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G8" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="18" t="n">
+      <c r="H8" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="20" t="n">
         <f aca="false">G8*H8</f>
         <v>8</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="J8" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="K8" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="L8" s="16" t="s">
+      <c r="L8" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M8" s="4" t="s">
+      <c r="M8" s="5" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G9" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="18" t="n">
+      <c r="H9" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="20" t="n">
         <f aca="false">G9*H9</f>
         <v>4</v>
       </c>
-      <c r="J9" s="4" t="s">
+      <c r="J9" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="K9" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="L9" s="16" t="s">
+      <c r="L9" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M9" s="4" t="s">
+      <c r="M9" s="5" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="G10" s="9" t="n">
+      <c r="G10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="18" t="n">
+      <c r="H10" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="20" t="n">
         <f aca="false">G10*H10</f>
         <v>15</v>
       </c>
-      <c r="J10" s="4" t="s">
+      <c r="J10" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="K10" s="4" t="s">
+      <c r="K10" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="L10" s="16" t="s">
+      <c r="L10" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="M10" s="4" t="s">
+      <c r="M10" s="5" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="G11" s="9" t="n">
+      <c r="G11" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="18" t="n">
+      <c r="H11" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="I11" s="19" t="n">
+      <c r="I11" s="20" t="n">
         <f aca="false">G11*H11</f>
         <v>25</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="J11" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="K11" s="4" t="s">
+      <c r="K11" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="L11" s="16" t="s">
+      <c r="L11" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="M11" s="4" t="s">
+      <c r="M11" s="5" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="G12" s="9" t="n">
+      <c r="G12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H12" s="18" t="n">
+      <c r="H12" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I12" s="19" t="n">
+      <c r="I12" s="20" t="n">
         <f aca="false">G12*H12</f>
         <v>8</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="J12" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="K12" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="L12" s="16" t="s">
+      <c r="L12" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="M12" s="5" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="G13" s="9" t="n">
+      <c r="G13" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="18" t="n">
+      <c r="H13" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="I13" s="19" t="n">
+      <c r="I13" s="20" t="n">
         <f aca="false">G13*H13</f>
         <v>8</v>
       </c>
-      <c r="J13" s="4" t="s">
+      <c r="J13" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="K13" s="4" t="s">
+      <c r="K13" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="L13" s="16" t="s">
+      <c r="L13" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M13" s="4" t="s">
+      <c r="M13" s="5" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="G14" s="9" t="n">
+      <c r="G14" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="18" t="n">
+      <c r="H14" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="I14" s="19" t="n">
+      <c r="I14" s="20" t="n">
         <f aca="false">G14*H14</f>
         <v>5</v>
       </c>
-      <c r="J14" s="4" t="s">
+      <c r="J14" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="K14" s="4" t="s">
+      <c r="K14" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="L14" s="16" t="s">
+      <c r="L14" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M14" s="4" t="s">
+      <c r="M14" s="5" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="G15" s="9" t="n">
+      <c r="G15" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="18" t="n">
+      <c r="H15" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="I15" s="19" t="n">
+      <c r="I15" s="20" t="n">
         <f aca="false">G15*H15</f>
         <v>3</v>
       </c>
-      <c r="J15" s="4" t="s">
+      <c r="J15" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="K15" s="4" t="s">
+      <c r="K15" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="L15" s="16" t="s">
+      <c r="L15" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M15" s="4" t="s">
+      <c r="M15" s="5" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="G16" s="9" t="n">
+      <c r="G16" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H16" s="18" t="n">
+      <c r="H16" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="I16" s="19" t="n">
+      <c r="I16" s="20" t="n">
         <f aca="false">G16*H16</f>
         <v>6</v>
       </c>
-      <c r="J16" s="4" t="s">
+      <c r="J16" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="K16" s="4" t="s">
+      <c r="K16" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="L16" s="16" t="s">
+      <c r="L16" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M16" s="4" t="s">
+      <c r="M16" s="5" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="G17" s="9" t="n">
+      <c r="G17" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H17" s="18" t="n">
+      <c r="H17" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="I17" s="19" t="n">
+      <c r="I17" s="20" t="n">
         <f aca="false">G17*H17</f>
         <v>4</v>
       </c>
-      <c r="J17" s="4" t="s">
+      <c r="J17" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="K17" s="4" t="s">
+      <c r="K17" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="L17" s="16" t="s">
+      <c r="L17" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M17" s="4" t="s">
+      <c r="M17" s="5" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="n">
+      <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="F18" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="G18" s="9" t="n">
+      <c r="G18" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H18" s="18" t="n">
+      <c r="H18" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="I18" s="19" t="n">
+      <c r="I18" s="20" t="n">
         <f aca="false">G18*H18</f>
         <v>3</v>
       </c>
-      <c r="J18" s="4" t="s">
+      <c r="J18" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="K18" s="4" t="s">
+      <c r="K18" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="L18" s="16" t="s">
+      <c r="L18" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M18" s="4"/>
+      <c r="M18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="F19" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="G19" s="9" t="n">
+      <c r="G19" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H19" s="18" t="n">
+      <c r="H19" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="I19" s="19" t="n">
+      <c r="I19" s="20" t="n">
         <f aca="false">G19*H19</f>
         <v>2</v>
       </c>
-      <c r="J19" s="4" t="s">
+      <c r="J19" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="K19" s="4" t="s">
+      <c r="K19" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="L19" s="16" t="s">
+      <c r="L19" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="M19" s="4" t="s">
+      <c r="M19" s="5" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="n">
+      <c r="A20" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="F20" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="G20" s="9" t="n">
+      <c r="G20" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H20" s="18" t="n">
+      <c r="H20" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="I20" s="19" t="n">
+      <c r="I20" s="20" t="n">
         <f aca="false">G20*H20</f>
         <v>2</v>
       </c>
-      <c r="J20" s="4" t="s">
+      <c r="J20" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="K20" s="4" t="s">
+      <c r="K20" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="L20" s="16" t="s">
+      <c r="L20" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="M20" s="4" t="s">
+      <c r="M20" s="5" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="F21" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="G21" s="9" t="n">
+      <c r="G21" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="18" t="n">
+      <c r="H21" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="I21" s="19" t="n">
+      <c r="I21" s="20" t="n">
         <f aca="false">G21*H21</f>
         <v>1</v>
       </c>
-      <c r="J21" s="4" t="s">
+      <c r="J21" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="K21" s="4" t="s">
+      <c r="K21" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="L21" s="16" t="s">
+      <c r="L21" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="M21" s="4" t="s">
+      <c r="M21" s="5" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="n">
+      <c r="A22" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F22" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="G22" s="9" t="n">
+      <c r="G22" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="18" t="n">
+      <c r="H22" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="I22" s="19" t="n">
+      <c r="I22" s="20" t="n">
         <f aca="false">G22*H22</f>
         <v>5</v>
       </c>
-      <c r="J22" s="4" t="s">
+      <c r="J22" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="K22" s="4" t="s">
+      <c r="K22" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="L22" s="16" t="s">
+      <c r="L22" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="M22" s="4" t="s">
+      <c r="M22" s="5" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="n">
+      <c r="A23" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F23" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="G23" s="9" t="n">
+      <c r="G23" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="18" t="n">
+      <c r="H23" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="I23" s="19" t="n">
+      <c r="I23" s="20" t="n">
         <f aca="false">G23*H23</f>
         <v>6</v>
       </c>
-      <c r="J23" s="4" t="s">
+      <c r="J23" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="K23" s="4" t="s">
+      <c r="K23" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="L23" s="16" t="s">
+      <c r="L23" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="M23" s="4" t="s">
+      <c r="M23" s="5" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="n">
+      <c r="A24" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="F24" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="G24" s="9" t="n">
+      <c r="G24" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H24" s="18" t="n">
+      <c r="H24" s="19" t="n">
         <v>20</v>
       </c>
-      <c r="I24" s="19" t="n">
+      <c r="I24" s="20" t="n">
         <f aca="false">G24*H24</f>
         <v>20</v>
       </c>
-      <c r="J24" s="4" t="s">
+      <c r="J24" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="K24" s="4" t="s">
+      <c r="K24" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="L24" s="16" t="s">
+      <c r="L24" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="M24" s="4" t="s">
+      <c r="M24" s="5" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H25" s="2" t="s">
+      <c r="H25" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="I25" s="20" t="n">
+      <c r="I25" s="21" t="n">
         <f aca="false">SUM(I5:I24)</f>
-        <v>153</v>
+        <v>143</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="4" t="s">
         <v>235</v>
       </c>
     </row>
@@ -3393,198 +3397,198 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="B3" s="21" t="n">
+      <c r="B3" s="22" t="n">
         <v>0.79</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="16" t="s">
         <v>239</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>240</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="16" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="23" t="n">
         <f aca="false">BOM!I5+BOM!I6</f>
-        <v>28</v>
-      </c>
-      <c r="C6" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="23" t="n">
         <f aca="false">SUM(BOM!I8:I11)</f>
         <v>52</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="B8" s="22" t="n">
+      <c r="B8" s="23" t="n">
         <f aca="false">SUM(BOM!I12:I13)</f>
         <v>16</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="23" t="n">
         <f aca="false">SUM(BOM!I14:I21)</f>
         <v>26</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="23" t="n">
         <f aca="false">BOM!I22</f>
         <v>5</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B11" s="23" t="n">
         <f aca="false">BOM!I23</f>
         <v>6</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="B12" s="22" t="n">
+      <c r="B12" s="23" t="n">
         <f aca="false">BOM!I24</f>
         <v>20</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="B13" s="20" t="n">
+      <c r="B13" s="21" t="n">
         <f aca="false">SUM(B6:B12)</f>
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="8" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="10" t="n">
         <v>0.75</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="B17" s="9" t="n">
+      <c r="B17" s="10" t="n">
         <v>1.55</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="B18" s="20" t="n">
+      <c r="B18" s="21" t="n">
         <f aca="false">B13*B16</f>
-        <v>114.75</v>
+        <v>105.75</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="B19" s="20" t="n">
+      <c r="B19" s="21" t="n">
         <f aca="false">B13*B17</f>
-        <v>237.15</v>
+        <v>218.55</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>261</v>
       </c>
     </row>
@@ -3605,168 +3609,168 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>262</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="B3" s="10" t="n">
+      <c r="B3" s="11" t="n">
         <f aca="false">70*280/100</f>
         <v>196</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>264</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>265</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="16" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>270</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>274</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>276</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>280</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="3" t="n">
         <f aca="false">SUM(B6:B12)</f>
         <v>160</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="3" t="n">
         <f aca="false">B3-B13</f>
         <v>36</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>284</v>
       </c>
     </row>
@@ -3787,374 +3791,374 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="16" t="s">
         <v>287</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="16" t="s">
         <v>239</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="16" t="s">
         <v>288</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="E4" s="15" t="s">
+      <c r="E4" s="16" t="s">
         <v>289</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="16" t="s">
         <v>290</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="16" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="17" t="s">
         <v>292</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>293</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="E5" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="F5" s="24" t="n">
+      <c r="F5" s="25" t="n">
         <f aca="false">D5*E5</f>
         <v>16</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="5" t="s">
         <v>294</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="H5" s="17" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="17" t="s">
         <v>296</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>297</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>298</v>
       </c>
-      <c r="D6" s="23" t="n">
+      <c r="D6" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E6" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="24" t="n">
+      <c r="F6" s="25" t="n">
         <f aca="false">D6*E6</f>
         <v>6</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="5" t="s">
         <v>299</v>
       </c>
-      <c r="H6" s="16" t="s">
+      <c r="H6" s="17" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="17" t="s">
         <v>300</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>301</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="24" t="n">
+      <c r="F7" s="25" t="n">
         <f aca="false">D7*E7</f>
         <v>12</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="H7" s="16" t="s">
+      <c r="H7" s="17" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="17" t="s">
         <v>304</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>305</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>306</v>
       </c>
-      <c r="D8" s="23" t="n">
+      <c r="D8" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="23" t="n">
+      <c r="E8" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="24" t="n">
+      <c r="F8" s="25" t="n">
         <f aca="false">D8*E8</f>
         <v>12</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="5" t="s">
         <v>307</v>
       </c>
-      <c r="H8" s="16" t="s">
+      <c r="H8" s="17" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="17" t="s">
         <v>308</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>309</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="23" t="n">
+      <c r="E9" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="24" t="n">
+      <c r="F9" s="25" t="n">
         <f aca="false">D9*E9</f>
         <v>12</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="5" t="s">
         <v>311</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="17" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="17" t="s">
         <v>312</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>314</v>
       </c>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E10" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="24" t="n">
+      <c r="F10" s="25" t="n">
         <f aca="false">D10*E10</f>
         <v>9</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="5" t="s">
         <v>315</v>
       </c>
-      <c r="H10" s="16" t="s">
+      <c r="H10" s="17" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="17" t="s">
         <v>316</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>317</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="D11" s="23" t="n">
+      <c r="D11" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="23" t="n">
+      <c r="E11" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="24" t="n">
+      <c r="F11" s="25" t="n">
         <f aca="false">D11*E11</f>
         <v>9</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="5" t="s">
         <v>319</v>
       </c>
-      <c r="H11" s="16" t="s">
+      <c r="H11" s="17" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="17" t="s">
         <v>320</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>321</v>
       </c>
-      <c r="D12" s="23" t="n">
+      <c r="D12" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="23" t="n">
+      <c r="E12" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="24" t="n">
+      <c r="F12" s="25" t="n">
         <f aca="false">D12*E12</f>
         <v>9</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="5" t="s">
         <v>322</v>
       </c>
-      <c r="H12" s="16" t="s">
+      <c r="H12" s="17" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="17" t="s">
         <v>323</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>324</v>
       </c>
-      <c r="D13" s="23" t="n">
+      <c r="D13" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="23" t="n">
+      <c r="E13" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F13" s="24" t="n">
+      <c r="F13" s="25" t="n">
         <f aca="false">D13*E13</f>
         <v>9</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="H13" s="16" t="s">
+      <c r="H13" s="17" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="17" t="s">
         <v>326</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>327</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>328</v>
       </c>
-      <c r="D14" s="23" t="n">
+      <c r="D14" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="23" t="n">
+      <c r="E14" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="24" t="n">
+      <c r="F14" s="25" t="n">
         <f aca="false">D14*E14</f>
         <v>6</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="H14" s="16" t="s">
+      <c r="H14" s="17" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="17" t="s">
         <v>330</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>331</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>332</v>
       </c>
-      <c r="D15" s="23" t="n">
+      <c r="D15" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="E15" s="23" t="n">
+      <c r="E15" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="24" t="n">
+      <c r="F15" s="25" t="n">
         <f aca="false">D15*E15</f>
         <v>6</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="H15" s="16" t="s">
+      <c r="H15" s="17" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="17" t="s">
         <v>334</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>336</v>
       </c>
-      <c r="D16" s="23" t="n">
+      <c r="D16" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="23" t="n">
+      <c r="E16" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="F16" s="24" t="n">
+      <c r="F16" s="25" t="n">
         <f aca="false">D16*E16</f>
         <v>6</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="H16" s="16" t="s">
+      <c r="H16" s="17" t="s">
         <v>295</v>
       </c>
     </row>
@@ -4175,226 +4179,226 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="16" t="s">
         <v>339</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="16" t="s">
         <v>340</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>343</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>344</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>346</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>347</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>348</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>349</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>350</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>351</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>352</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>353</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>354</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>355</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>356</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>357</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>358</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>359</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>360</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>362</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>363</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="5" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>365</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>366</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="5" t="s">
         <v>367</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>368</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>369</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="5" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="5" t="s">
         <v>372</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="5" t="s">
         <v>232</v>
       </c>
     </row>

</xml_diff>